<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_regionales_sexo_edad)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_sexo_edad/plot_historia_nacional_i_ingr_a_2018_nacional.xlsx
+++ b/output/graficos_regionales_sexo_edad/plot_historia_nacional_i_ingr_a_2018_nacional.xlsx
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-18 09:02</t>
+    <t xml:space="preserve">2026-10-05 04:35</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -796,7 +796,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>620781.12</v>
+        <v>620781.13</v>
       </c>
     </row>
     <row r="9">
@@ -917,7 +917,7 @@
         <v>20</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1116003.62</v>
+        <v>1116003.63</v>
       </c>
     </row>
     <row r="20">
@@ -939,7 +939,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1370522.12</v>
+        <v>1370522.13</v>
       </c>
     </row>
     <row r="22">
@@ -950,7 +950,7 @@
         <v>20</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1449180.12</v>
+        <v>1449180.13</v>
       </c>
     </row>
     <row r="23">
@@ -994,7 +994,7 @@
         <v>21</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1052891.62</v>
+        <v>1052891.63</v>
       </c>
     </row>
     <row r="27">
@@ -1027,7 +1027,7 @@
         <v>21</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1435887.12</v>
+        <v>1435887.13</v>
       </c>
     </row>
     <row r="30">
@@ -1093,7 +1093,7 @@
         <v>22</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>1168320.12</v>
+        <v>1168320.13</v>
       </c>
     </row>
     <row r="36">

</xml_diff>